<commit_message>
Updated Power BI report and READ me file with latest changes
</commit_message>
<xml_diff>
--- a/Data/Singapore average annual expenditure (Import).xlsx
+++ b/Data/Singapore average annual expenditure (Import).xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Afiqr\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Afiqr\Downloads\Power BI Dashboards\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF662C78-1BFF-44D1-8971-E66F41430AA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB6AE772-FDB0-4B95-81E4-C5117C729255}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="3" activeTab="3" xr2:uid="{EDD3299F-02BD-44B7-B90A-9F08C3E22831}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{EDD3299F-02BD-44B7-B90A-9F08C3E22831}"/>
   </bookViews>
   <sheets>
     <sheet name="Average monthly expenditure per" sheetId="2" r:id="rId1"/>
@@ -741,7 +741,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -880,9 +880,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1796,217 +1793,297 @@
     </dxf>
     <dxf>
       <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+      <border diagonalUp="0" diagonalDown="0">
         <left/>
         <right/>
         <top style="thin">
           <color theme="4" tint="0.39997558519241921"/>
         </top>
         <bottom/>
+        <vertical/>
+        <horizontal/>
       </border>
     </dxf>
     <dxf>
       <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+      <border diagonalUp="0" diagonalDown="0">
         <left/>
         <right/>
         <top style="thin">
           <color theme="4" tint="0.39997558519241921"/>
         </top>
         <bottom/>
+        <vertical/>
+        <horizontal/>
       </border>
     </dxf>
     <dxf>
       <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+      <border diagonalUp="0" diagonalDown="0">
         <left/>
         <right/>
         <top style="thin">
           <color theme="4" tint="0.39997558519241921"/>
         </top>
         <bottom/>
+        <vertical/>
+        <horizontal/>
       </border>
     </dxf>
     <dxf>
       <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+      <border diagonalUp="0" diagonalDown="0">
         <left/>
         <right/>
         <top style="thin">
           <color theme="4" tint="0.39997558519241921"/>
         </top>
         <bottom/>
+        <vertical/>
+        <horizontal/>
       </border>
     </dxf>
     <dxf>
       <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+      <border diagonalUp="0" diagonalDown="0">
         <left/>
         <right/>
         <top style="thin">
           <color theme="4" tint="0.39997558519241921"/>
         </top>
         <bottom/>
+        <vertical/>
+        <horizontal/>
       </border>
     </dxf>
     <dxf>
       <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+      <border diagonalUp="0" diagonalDown="0">
         <left/>
         <right/>
         <top style="thin">
           <color theme="4" tint="0.39997558519241921"/>
         </top>
         <bottom/>
+        <vertical/>
+        <horizontal/>
       </border>
     </dxf>
     <dxf>
       <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+      <border diagonalUp="0" diagonalDown="0">
         <left/>
         <right/>
         <top style="thin">
           <color theme="4" tint="0.39997558519241921"/>
         </top>
         <bottom/>
+        <vertical/>
+        <horizontal/>
       </border>
     </dxf>
     <dxf>
       <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+      <border diagonalUp="0" diagonalDown="0">
         <left/>
         <right/>
         <top style="thin">
           <color theme="4" tint="0.39997558519241921"/>
         </top>
         <bottom/>
+        <vertical/>
+        <horizontal/>
       </border>
     </dxf>
     <dxf>
       <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+      <border diagonalUp="0" diagonalDown="0">
         <left/>
         <right/>
         <top style="thin">
           <color theme="4" tint="0.39997558519241921"/>
         </top>
         <bottom/>
+        <vertical/>
+        <horizontal/>
       </border>
     </dxf>
     <dxf>
       <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+      <border diagonalUp="0" diagonalDown="0">
         <left/>
         <right/>
         <top style="thin">
           <color theme="4" tint="0.39997558519241921"/>
         </top>
         <bottom/>
+        <vertical/>
+        <horizontal/>
       </border>
     </dxf>
     <dxf>
       <font>
-        <b/>
+        <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
         <condense val="0"/>
@@ -2017,44 +2094,46 @@
         <vertAlign val="baseline"/>
         <sz val="11"/>
         <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </left>
         <right/>
         <top style="thin">
           <color theme="4" tint="0.39997558519241921"/>
         </top>
         <bottom/>
+        <vertical/>
+        <horizontal/>
       </border>
     </dxf>
     <dxf>
       <border outline="0">
-        <left style="thin">
+        <right style="thin">
           <color theme="4" tint="0.39997558519241921"/>
-        </left>
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
+        </right>
       </border>
     </dxf>
     <dxf>
       <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
       </font>
     </dxf>
     <dxf>
@@ -2069,203 +2148,17 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="11"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
+        <color theme="0"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
       </font>
       <fill>
         <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.79998168889431442"/>
-          <bgColor theme="4" tint="0.79998168889431442"/>
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
         </patternFill>
       </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <border outline="0">
@@ -2713,297 +2606,217 @@
     </dxf>
     <dxf>
       <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-      <border diagonalUp="0" diagonalDown="0">
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left/>
         <right/>
         <top style="thin">
           <color theme="4" tint="0.39997558519241921"/>
         </top>
         <bottom/>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
       <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-      <border diagonalUp="0" diagonalDown="0">
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left/>
         <right/>
         <top style="thin">
           <color theme="4" tint="0.39997558519241921"/>
         </top>
         <bottom/>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
       <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-      <border diagonalUp="0" diagonalDown="0">
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left/>
         <right/>
         <top style="thin">
           <color theme="4" tint="0.39997558519241921"/>
         </top>
         <bottom/>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
       <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-      <border diagonalUp="0" diagonalDown="0">
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left/>
         <right/>
         <top style="thin">
           <color theme="4" tint="0.39997558519241921"/>
         </top>
         <bottom/>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
       <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-      <border diagonalUp="0" diagonalDown="0">
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left/>
         <right/>
         <top style="thin">
           <color theme="4" tint="0.39997558519241921"/>
         </top>
         <bottom/>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
       <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-      <border diagonalUp="0" diagonalDown="0">
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left/>
         <right/>
         <top style="thin">
           <color theme="4" tint="0.39997558519241921"/>
         </top>
         <bottom/>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
       <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-      <border diagonalUp="0" diagonalDown="0">
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left/>
         <right/>
         <top style="thin">
           <color theme="4" tint="0.39997558519241921"/>
         </top>
         <bottom/>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
       <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-      <border diagonalUp="0" diagonalDown="0">
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left/>
         <right/>
         <top style="thin">
           <color theme="4" tint="0.39997558519241921"/>
         </top>
         <bottom/>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
       <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-      <border diagonalUp="0" diagonalDown="0">
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left/>
         <right/>
         <top style="thin">
           <color theme="4" tint="0.39997558519241921"/>
         </top>
         <bottom/>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
       <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-      <border diagonalUp="0" diagonalDown="0">
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
         <left/>
         <right/>
         <top style="thin">
           <color theme="4" tint="0.39997558519241921"/>
         </top>
         <bottom/>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
       <font>
-        <b val="0"/>
+        <b/>
         <i val="0"/>
         <strike val="0"/>
         <condense val="0"/>
@@ -3014,33 +2827,49 @@
         <vertAlign val="baseline"/>
         <sz val="11"/>
         <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </left>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
         <right/>
         <top style="thin">
           <color theme="4" tint="0.39997558519241921"/>
         </top>
         <bottom/>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
       <border outline="0">
-        <right style="thin">
+        <left style="thin">
           <color theme="4" tint="0.39997558519241921"/>
-        </right>
+        </left>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
       </border>
     </dxf>
     <dxf>
       <font>
-        <b val="0"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
         <i val="0"/>
         <strike val="0"/>
         <condense val="0"/>
@@ -3050,35 +2879,203 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="0"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
       </font>
       <fill>
         <patternFill patternType="solid">
-          <fgColor theme="4"/>
-          <bgColor theme="4"/>
+          <fgColor theme="4" tint="0.79998168889431442"/>
+          <bgColor theme="4" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -3131,21 +3128,21 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B580B91D-BA53-429E-B650-7B9F842A3154}" name="Table1" displayName="Table1" ref="B3:M21" totalsRowShown="0" headerRowDxfId="100" dataDxfId="99" tableBorderDxfId="98">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B580B91D-BA53-429E-B650-7B9F842A3154}" name="Table1" displayName="Table1" ref="B3:M21" totalsRowShown="0" headerRowDxfId="86" dataDxfId="85" tableBorderDxfId="84">
   <autoFilter ref="B3:M21" xr:uid="{B580B91D-BA53-429E-B650-7B9F842A3154}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{1EC5AC4F-7874-43B3-A125-03DBD49C54AC}" name="Country" dataDxfId="97"/>
-    <tableColumn id="2" xr3:uid="{BFFAB26E-0E02-405C-906F-6041DED128A1}" name="Type of expenditure/ data" dataDxfId="96"/>
-    <tableColumn id="3" xr3:uid="{FB285517-1C77-44D6-AB23-6D4ECC58DD7B}" name="2015" dataDxfId="95"/>
-    <tableColumn id="4" xr3:uid="{3784ACBC-DC31-4E6B-9F1A-EFE822281DCE}" name="2016" dataDxfId="94"/>
-    <tableColumn id="5" xr3:uid="{0E56797C-8F9C-4132-B0C0-890AC9B99416}" name="2017" dataDxfId="93"/>
-    <tableColumn id="6" xr3:uid="{9F1DA9EB-1DE1-4B8C-84A4-5112447128B3}" name="2018" dataDxfId="92"/>
-    <tableColumn id="7" xr3:uid="{79B724F3-F3C0-4EBC-BDDA-4A109F83BDFA}" name="2019" dataDxfId="91"/>
-    <tableColumn id="8" xr3:uid="{793A16FA-A9C1-4EBD-B58A-98B9415432F5}" name="2020" dataDxfId="90"/>
-    <tableColumn id="9" xr3:uid="{8BC61902-1AF9-43B8-9AD4-261CC3FF7B00}" name="2021" dataDxfId="89"/>
-    <tableColumn id="10" xr3:uid="{9923BA07-93B5-4EE0-8C2A-A414726FCCAD}" name="2022" dataDxfId="88"/>
-    <tableColumn id="11" xr3:uid="{3311C278-8A39-439E-9D23-8FFA0583D47E}" name="2023" dataDxfId="87"/>
-    <tableColumn id="12" xr3:uid="{2A83443B-47FE-4F4B-84C6-D38731C26D0D}" name="2024" dataDxfId="86"/>
+    <tableColumn id="1" xr3:uid="{1EC5AC4F-7874-43B3-A125-03DBD49C54AC}" name="Country" dataDxfId="83"/>
+    <tableColumn id="2" xr3:uid="{BFFAB26E-0E02-405C-906F-6041DED128A1}" name="Type of expenditure/ data" dataDxfId="82"/>
+    <tableColumn id="3" xr3:uid="{FB285517-1C77-44D6-AB23-6D4ECC58DD7B}" name="2015" dataDxfId="81"/>
+    <tableColumn id="4" xr3:uid="{3784ACBC-DC31-4E6B-9F1A-EFE822281DCE}" name="2016" dataDxfId="80"/>
+    <tableColumn id="5" xr3:uid="{0E56797C-8F9C-4132-B0C0-890AC9B99416}" name="2017" dataDxfId="79"/>
+    <tableColumn id="6" xr3:uid="{9F1DA9EB-1DE1-4B8C-84A4-5112447128B3}" name="2018" dataDxfId="78"/>
+    <tableColumn id="7" xr3:uid="{79B724F3-F3C0-4EBC-BDDA-4A109F83BDFA}" name="2019" dataDxfId="77"/>
+    <tableColumn id="8" xr3:uid="{793A16FA-A9C1-4EBD-B58A-98B9415432F5}" name="2020" dataDxfId="76"/>
+    <tableColumn id="9" xr3:uid="{8BC61902-1AF9-43B8-9AD4-261CC3FF7B00}" name="2021" dataDxfId="75"/>
+    <tableColumn id="10" xr3:uid="{9923BA07-93B5-4EE0-8C2A-A414726FCCAD}" name="2022" dataDxfId="74"/>
+    <tableColumn id="11" xr3:uid="{3311C278-8A39-439E-9D23-8FFA0583D47E}" name="2023" dataDxfId="73"/>
+    <tableColumn id="12" xr3:uid="{2A83443B-47FE-4F4B-84C6-D38731C26D0D}" name="2024" dataDxfId="72"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3169,23 +3166,23 @@
   <autoFilter ref="B2:L5" xr:uid="{4FEFB451-4FEE-4A19-BA27-C2BC501F2342}"/>
   <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{C8AA0414-2898-4FD6-A531-4C4308E68748}" name="Type of Expenditure"/>
-    <tableColumn id="2" xr3:uid="{FC3D0AE4-1D5B-4262-B9C7-4DB2CF30F3D8}" name="2015" dataDxfId="85"/>
-    <tableColumn id="3" xr3:uid="{35D74E1E-2E23-4526-A171-27A7FF1E41BE}" name="2016" dataDxfId="84"/>
-    <tableColumn id="4" xr3:uid="{F423909A-A134-4401-B6F6-6D3578DDCFD5}" name="2017" dataDxfId="83"/>
-    <tableColumn id="5" xr3:uid="{3327740A-9844-434B-AD7D-746AE9FD9775}" name="2018" dataDxfId="82"/>
-    <tableColumn id="6" xr3:uid="{DB96F0A6-D2F4-44BF-B7DA-3CC97EEF7B5D}" name="2019" dataDxfId="81"/>
-    <tableColumn id="7" xr3:uid="{E0D17029-1150-445A-80B0-3D4D9E4DCA01}" name="2020" dataDxfId="80"/>
-    <tableColumn id="8" xr3:uid="{8CB5D131-BFF7-49F9-A8FC-A651342E3DE4}" name="2021" dataDxfId="79"/>
-    <tableColumn id="9" xr3:uid="{7D9D9BF3-D5F1-4D9C-8F52-4FFC211BD394}" name="2022" dataDxfId="78"/>
-    <tableColumn id="10" xr3:uid="{5031A11C-FA78-42FB-919A-573EB69BBC10}" name="2023" dataDxfId="77"/>
-    <tableColumn id="11" xr3:uid="{A95E1EC7-9C3D-4090-9AE1-55E0EF32E0B8}" name="2024" dataDxfId="76"/>
+    <tableColumn id="2" xr3:uid="{FC3D0AE4-1D5B-4262-B9C7-4DB2CF30F3D8}" name="2015" dataDxfId="71"/>
+    <tableColumn id="3" xr3:uid="{35D74E1E-2E23-4526-A171-27A7FF1E41BE}" name="2016" dataDxfId="70"/>
+    <tableColumn id="4" xr3:uid="{F423909A-A134-4401-B6F6-6D3578DDCFD5}" name="2017" dataDxfId="69"/>
+    <tableColumn id="5" xr3:uid="{3327740A-9844-434B-AD7D-746AE9FD9775}" name="2018" dataDxfId="68"/>
+    <tableColumn id="6" xr3:uid="{DB96F0A6-D2F4-44BF-B7DA-3CC97EEF7B5D}" name="2019" dataDxfId="67"/>
+    <tableColumn id="7" xr3:uid="{E0D17029-1150-445A-80B0-3D4D9E4DCA01}" name="2020" dataDxfId="66"/>
+    <tableColumn id="8" xr3:uid="{8CB5D131-BFF7-49F9-A8FC-A651342E3DE4}" name="2021" dataDxfId="65"/>
+    <tableColumn id="9" xr3:uid="{7D9D9BF3-D5F1-4D9C-8F52-4FFC211BD394}" name="2022" dataDxfId="64"/>
+    <tableColumn id="10" xr3:uid="{5031A11C-FA78-42FB-919A-573EB69BBC10}" name="2023" dataDxfId="63"/>
+    <tableColumn id="11" xr3:uid="{A95E1EC7-9C3D-4090-9AE1-55E0EF32E0B8}" name="2024" dataDxfId="62"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{11E50511-12E8-4D3B-9CC3-5CD389AD9D4B}" name="Table9" displayName="Table9" ref="B9:M12" totalsRowShown="0" headerRowDxfId="75" tableBorderDxfId="74">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{11E50511-12E8-4D3B-9CC3-5CD389AD9D4B}" name="Table9" displayName="Table9" ref="B9:M12" totalsRowShown="0" headerRowDxfId="61" tableBorderDxfId="60">
   <autoFilter ref="B9:M12" xr:uid="{11E50511-12E8-4D3B-9CC3-5CD389AD9D4B}"/>
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{E0AB75B4-C5D8-43C4-B84F-3B212FF42F96}" name="Coutry"/>
@@ -3206,80 +3203,80 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{BD1E9208-3713-421C-8720-40BEAEE4603D}" name="Table11" displayName="Table11" ref="B2:M10" totalsRowShown="0" headerRowDxfId="114" dataDxfId="113" tableBorderDxfId="112">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{BD1E9208-3713-421C-8720-40BEAEE4603D}" name="Table11" displayName="Table11" ref="B2:M10" totalsRowShown="0" headerRowDxfId="59" dataDxfId="58" tableBorderDxfId="57">
   <autoFilter ref="B2:M10" xr:uid="{BD1E9208-3713-421C-8720-40BEAEE4603D}"/>
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{A54EC52C-57AC-4B9B-A17E-254AD0FECE46}" name="Country"/>
-    <tableColumn id="2" xr3:uid="{9D546B6D-1BA8-4572-9FFC-76A7B21A20E3}" name="Tyoe of Data" dataDxfId="111"/>
-    <tableColumn id="3" xr3:uid="{0E6E8A7C-8A21-4239-8D64-D0BE53B1347C}" name="2015" dataDxfId="110"/>
-    <tableColumn id="4" xr3:uid="{C0753B09-1D94-4404-89E2-C7D394930302}" name="2016" dataDxfId="109"/>
-    <tableColumn id="5" xr3:uid="{765A992C-0B73-4AAC-A8CD-28AFCCA8E6EC}" name="2017" dataDxfId="108"/>
-    <tableColumn id="6" xr3:uid="{C2A7FAB1-911B-4179-90A9-907581DD5E81}" name="2018" dataDxfId="107"/>
-    <tableColumn id="7" xr3:uid="{2CD059E7-8D26-4D6B-AFA5-722490DD39DA}" name="2019" dataDxfId="106"/>
-    <tableColumn id="8" xr3:uid="{CFAAE1C5-939A-4805-858D-E9EE0E32D08E}" name="2020" dataDxfId="105"/>
-    <tableColumn id="9" xr3:uid="{643F5E59-171E-49CB-817A-FCBCA93E5B15}" name="2021" dataDxfId="104"/>
-    <tableColumn id="10" xr3:uid="{19F06651-3EC0-4A00-ABFC-A5DB3F81629B}" name="2022" dataDxfId="103"/>
-    <tableColumn id="11" xr3:uid="{7545C349-0D3E-439D-9D0A-8458B089EA86}" name="2023" dataDxfId="102"/>
-    <tableColumn id="12" xr3:uid="{FB43D416-C26C-4DCA-BA01-A3A2DF0DC787}" name="2024" dataDxfId="101"/>
+    <tableColumn id="2" xr3:uid="{9D546B6D-1BA8-4572-9FFC-76A7B21A20E3}" name="Tyoe of Data" dataDxfId="56"/>
+    <tableColumn id="3" xr3:uid="{0E6E8A7C-8A21-4239-8D64-D0BE53B1347C}" name="2015" dataDxfId="55"/>
+    <tableColumn id="4" xr3:uid="{C0753B09-1D94-4404-89E2-C7D394930302}" name="2016" dataDxfId="54"/>
+    <tableColumn id="5" xr3:uid="{765A992C-0B73-4AAC-A8CD-28AFCCA8E6EC}" name="2017" dataDxfId="53"/>
+    <tableColumn id="6" xr3:uid="{C2A7FAB1-911B-4179-90A9-907581DD5E81}" name="2018" dataDxfId="52"/>
+    <tableColumn id="7" xr3:uid="{2CD059E7-8D26-4D6B-AFA5-722490DD39DA}" name="2019" dataDxfId="51"/>
+    <tableColumn id="8" xr3:uid="{CFAAE1C5-939A-4805-858D-E9EE0E32D08E}" name="2020" dataDxfId="50"/>
+    <tableColumn id="9" xr3:uid="{643F5E59-171E-49CB-817A-FCBCA93E5B15}" name="2021" dataDxfId="49"/>
+    <tableColumn id="10" xr3:uid="{19F06651-3EC0-4A00-ABFC-A5DB3F81629B}" name="2022" dataDxfId="48"/>
+    <tableColumn id="11" xr3:uid="{7545C349-0D3E-439D-9D0A-8458B089EA86}" name="2023" dataDxfId="47"/>
+    <tableColumn id="12" xr3:uid="{FB43D416-C26C-4DCA-BA01-A3A2DF0DC787}" name="2024" dataDxfId="46"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{C3FDDCB7-65A5-4BB9-9220-3F6843716D53}" name="Table10" displayName="Table10" ref="B3:M5" tableType="queryTable" totalsRowShown="0" headerRowDxfId="73" dataDxfId="72">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{C3FDDCB7-65A5-4BB9-9220-3F6843716D53}" name="Table10" displayName="Table10" ref="B3:M5" tableType="queryTable" totalsRowShown="0" headerRowDxfId="114" dataDxfId="113">
   <autoFilter ref="B3:M5" xr:uid="{C3FDDCB7-65A5-4BB9-9220-3F6843716D53}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{DFD6FB3E-6BF4-4F3A-A63A-E058271AE34A}" uniqueName="1" name="Year" queryTableFieldId="1" dataDxfId="71"/>
-    <tableColumn id="16" xr3:uid="{14FE4773-3E84-431F-AEE5-1420D81F1AD7}" uniqueName="16" name="2014" queryTableFieldId="16" dataDxfId="70"/>
-    <tableColumn id="17" xr3:uid="{AC0CF2F5-F292-4412-A69D-2A89668FA811}" uniqueName="17" name="2015" queryTableFieldId="17" dataDxfId="69"/>
-    <tableColumn id="18" xr3:uid="{55BF3E8C-8DFD-4472-9793-103A4BC0C327}" uniqueName="18" name="2016" queryTableFieldId="18" dataDxfId="68"/>
-    <tableColumn id="19" xr3:uid="{DEFB5C65-B2C6-4057-9F38-78BA29F1FF40}" uniqueName="19" name="2017" queryTableFieldId="19" dataDxfId="67"/>
-    <tableColumn id="20" xr3:uid="{C3FC9CA6-AF92-44A3-80DD-266C26C03741}" uniqueName="20" name="2018" queryTableFieldId="20" dataDxfId="66"/>
-    <tableColumn id="21" xr3:uid="{656476D9-A870-45F1-8B01-EC1A99FF7627}" uniqueName="21" name="2019" queryTableFieldId="21" dataDxfId="65"/>
-    <tableColumn id="22" xr3:uid="{503CD6F8-DEB7-4596-9ACA-C13656883920}" uniqueName="22" name="2020" queryTableFieldId="22" dataDxfId="64"/>
-    <tableColumn id="23" xr3:uid="{570D3573-A02A-41A3-AEB3-175721101469}" uniqueName="23" name="2021" queryTableFieldId="23" dataDxfId="63"/>
-    <tableColumn id="24" xr3:uid="{7C4F4421-B314-42EC-B133-85519B025B44}" uniqueName="24" name="2022" queryTableFieldId="24" dataDxfId="62"/>
-    <tableColumn id="25" xr3:uid="{13795E6D-E5C7-4563-8ECD-9951D9D290C5}" uniqueName="25" name="2023" queryTableFieldId="25" dataDxfId="61"/>
-    <tableColumn id="26" xr3:uid="{D3FF38A2-4153-499A-BF21-38A60F1B5525}" uniqueName="26" name="2024" queryTableFieldId="26" dataDxfId="60"/>
+    <tableColumn id="1" xr3:uid="{DFD6FB3E-6BF4-4F3A-A63A-E058271AE34A}" uniqueName="1" name="Year" queryTableFieldId="1" dataDxfId="112"/>
+    <tableColumn id="16" xr3:uid="{14FE4773-3E84-431F-AEE5-1420D81F1AD7}" uniqueName="16" name="2014" queryTableFieldId="16" dataDxfId="111"/>
+    <tableColumn id="17" xr3:uid="{AC0CF2F5-F292-4412-A69D-2A89668FA811}" uniqueName="17" name="2015" queryTableFieldId="17" dataDxfId="110"/>
+    <tableColumn id="18" xr3:uid="{55BF3E8C-8DFD-4472-9793-103A4BC0C327}" uniqueName="18" name="2016" queryTableFieldId="18" dataDxfId="109"/>
+    <tableColumn id="19" xr3:uid="{DEFB5C65-B2C6-4057-9F38-78BA29F1FF40}" uniqueName="19" name="2017" queryTableFieldId="19" dataDxfId="108"/>
+    <tableColumn id="20" xr3:uid="{C3FC9CA6-AF92-44A3-80DD-266C26C03741}" uniqueName="20" name="2018" queryTableFieldId="20" dataDxfId="107"/>
+    <tableColumn id="21" xr3:uid="{656476D9-A870-45F1-8B01-EC1A99FF7627}" uniqueName="21" name="2019" queryTableFieldId="21" dataDxfId="106"/>
+    <tableColumn id="22" xr3:uid="{503CD6F8-DEB7-4596-9ACA-C13656883920}" uniqueName="22" name="2020" queryTableFieldId="22" dataDxfId="105"/>
+    <tableColumn id="23" xr3:uid="{570D3573-A02A-41A3-AEB3-175721101469}" uniqueName="23" name="2021" queryTableFieldId="23" dataDxfId="104"/>
+    <tableColumn id="24" xr3:uid="{7C4F4421-B314-42EC-B133-85519B025B44}" uniqueName="24" name="2022" queryTableFieldId="24" dataDxfId="103"/>
+    <tableColumn id="25" xr3:uid="{13795E6D-E5C7-4563-8ECD-9951D9D290C5}" uniqueName="25" name="2023" queryTableFieldId="25" dataDxfId="102"/>
+    <tableColumn id="26" xr3:uid="{D3FF38A2-4153-499A-BF21-38A60F1B5525}" uniqueName="26" name="2024" queryTableFieldId="26" dataDxfId="101"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{E1F4BB61-04AA-4900-9E0A-082DB836C9BF}" name="Table4" displayName="Table4" ref="B8:L9" totalsRowShown="0" headerRowDxfId="59" dataDxfId="58" tableBorderDxfId="57">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{E1F4BB61-04AA-4900-9E0A-082DB836C9BF}" name="Table4" displayName="Table4" ref="B8:L9" totalsRowShown="0" headerRowDxfId="100" dataDxfId="99" tableBorderDxfId="98">
   <autoFilter ref="B8:L9" xr:uid="{E1F4BB61-04AA-4900-9E0A-082DB836C9BF}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{BB8BD6D7-53CD-4BC3-B989-CEF5D69AFB52}" name="Year" dataDxfId="56"/>
-    <tableColumn id="2" xr3:uid="{D0FD0292-2D39-42E5-B582-E71FA8BB10D1}" name="2015" dataDxfId="55">
+    <tableColumn id="1" xr3:uid="{BB8BD6D7-53CD-4BC3-B989-CEF5D69AFB52}" name="Year" dataDxfId="97"/>
+    <tableColumn id="2" xr3:uid="{D0FD0292-2D39-42E5-B582-E71FA8BB10D1}" name="2015" dataDxfId="96">
       <calculatedColumnFormula>(D4-C4)/C4</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{CA338C20-4263-4E75-AAD4-D11E8D19C920}" name="2016" dataDxfId="54">
+    <tableColumn id="3" xr3:uid="{CA338C20-4263-4E75-AAD4-D11E8D19C920}" name="2016" dataDxfId="95">
       <calculatedColumnFormula>(E4-D4)/D4</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{70193156-3F63-4D00-9599-6CE26FA15B32}" name="2017" dataDxfId="53">
+    <tableColumn id="4" xr3:uid="{70193156-3F63-4D00-9599-6CE26FA15B32}" name="2017" dataDxfId="94">
       <calculatedColumnFormula>(F4-E4)/E4</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{C877CECB-D042-43FD-A527-CD312745F9B7}" name="2018" dataDxfId="52">
+    <tableColumn id="5" xr3:uid="{C877CECB-D042-43FD-A527-CD312745F9B7}" name="2018" dataDxfId="93">
       <calculatedColumnFormula>(G4-F4)/F4</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{FA44D971-5177-4B57-9ACC-DB882C0F0AD5}" name="2019" dataDxfId="51">
+    <tableColumn id="6" xr3:uid="{FA44D971-5177-4B57-9ACC-DB882C0F0AD5}" name="2019" dataDxfId="92">
       <calculatedColumnFormula>(H4-G4)/G4</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{DACB31EB-904B-4C5B-967C-96BA42D78139}" name="2020" dataDxfId="50">
+    <tableColumn id="7" xr3:uid="{DACB31EB-904B-4C5B-967C-96BA42D78139}" name="2020" dataDxfId="91">
       <calculatedColumnFormula>(I4-H4)/H4</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{47B4F972-FBC3-4254-80AD-07396C21227B}" name="2021" dataDxfId="49">
+    <tableColumn id="8" xr3:uid="{47B4F972-FBC3-4254-80AD-07396C21227B}" name="2021" dataDxfId="90">
       <calculatedColumnFormula>(J4-I4)/I4</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{A309E90C-FAAC-4096-A499-E34B6974FD25}" name="2022" dataDxfId="48">
+    <tableColumn id="9" xr3:uid="{A309E90C-FAAC-4096-A499-E34B6974FD25}" name="2022" dataDxfId="89">
       <calculatedColumnFormula>(K4-J4)/J4</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{B14905D5-7680-4827-827B-E6FB916B74E6}" name="2023" dataDxfId="47">
+    <tableColumn id="10" xr3:uid="{B14905D5-7680-4827-827B-E6FB916B74E6}" name="2023" dataDxfId="88">
       <calculatedColumnFormula>(L4-K4)/K4</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{C9676F92-6E50-4DFE-AF59-63E65400728D}" name="2024" dataDxfId="46">
+    <tableColumn id="11" xr3:uid="{C9676F92-6E50-4DFE-AF59-63E65400728D}" name="2024" dataDxfId="87">
       <calculatedColumnFormula>(M4-L4)/L4</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -5169,7 +5166,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A1" s="74"/>
+      <c r="A1" s="19"/>
       <c r="O1" s="1" t="s">
         <v>82</v>
       </c>
@@ -5423,7 +5420,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" x14ac:dyDescent="0.35">
-      <c r="A1" s="74"/>
+      <c r="A1" s="19"/>
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.35">
       <c r="B2" s="26" t="s">
@@ -6084,7 +6081,7 @@
       <c r="A1" s="40" t="s">
         <v>52</v>
       </c>
-      <c r="D1" s="74"/>
+      <c r="D1" s="19"/>
     </row>
     <row r="3" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
       <c r="C3" s="41" t="s">
@@ -6403,7 +6400,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.35">
-      <c r="A1" s="74"/>
+      <c r="A1" s="19"/>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.35">
       <c r="B2" s="26" t="s">
@@ -6700,7 +6697,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A1" s="74"/>
+      <c r="A1" s="19"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B2" s="21" t="s">

</xml_diff>